<commit_message>
Matin londonien complet (07:12-09:28 UTC) : chiffres et grille Excel mis a jour
</commit_message>
<xml_diff>
--- a/reports/otc_clip_pricer.xlsx
+++ b/reports/otc_clip_pricer.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>IF($B$5="BTC",83874.82,2531.41)</f>
+        <f>IF($B$5="BTC",83360.83,2506.28)</f>
         <v/>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B16">
-        <f>IF(ISNUMBER(MATCH($B$5&amp;"|ALL3|"&amp;IF(AND($B$8&gt;=7,$B$8&lt;12),"London morning",IF(AND($B$8&gt;=12,$B$8&lt;16),"London + New York",IF(AND($B$8&gt;=16,$B$8&lt;21),"New York afternoon","All measured"))),'Sweep costs'!$A$2:$A$17,0)),IF(AND($B$8&gt;=7,$B$8&lt;12),"London morning",IF(AND($B$8&gt;=12,$B$8&lt;16),"London + New York",IF(AND($B$8&gt;=16,$B$8&lt;21),"New York afternoon","All measured"))),"All measured")</f>
+        <f>IF(ISNUMBER(MATCH($B$5&amp;"|ALL3|"&amp;IF(AND($B$8&gt;=7,$B$8&lt;12),"London morning",IF(AND($B$8&gt;=12,$B$8&lt;16),"London + New York",IF(AND($B$8&gt;=16,$B$8&lt;21),"New York afternoon","All measured"))),'Sweep costs'!$A$2:$A$25,0)),IF(AND($B$8&gt;=7,$B$8&lt;12),"London morning",IF(AND($B$8&gt;=12,$B$8&lt;16),"London + New York",IF(AND($B$8&gt;=16,$B$8&lt;21),"New York afternoon","All measured"))),"All measured")</f>
         <v/>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>INDEX('Sweep costs'!$F$2:$K$17,MATCH(B17,'Sweep costs'!$A$2:$A$17,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$17,MATCH(B17,'Sweep costs'!$A$2:$A$17,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$17,MATCH(B17,'Sweep costs'!$A$2:$A$17,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18))</f>
+        <f>INDEX('Sweep costs'!$F$2:$K$25,MATCH(B17,'Sweep costs'!$A$2:$A$25,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$25,MATCH(B17,'Sweep costs'!$A$2:$A$25,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$25,MATCH(B17,'Sweep costs'!$A$2:$A$25,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18))</f>
         <v/>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>MIN(INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)),INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)),INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$17,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$17,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)))</f>
+        <f>MIN(INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|binance|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)),INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|coinbase|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)),INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18)+(MAX(0.1,MIN(10,$B$7))-INDEX('Sweep costs'!$F$1:$K$1,1,B18))*(INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18+1)-INDEX('Sweep costs'!$F$2:$K$25,MATCH($B$5&amp;"|kraken|"&amp;B16,'Sweep costs'!$A$2:$A$25,0),B18))/(INDEX('Sweep costs'!$F$1:$K$1,1,B18+1)-INDEX('Sweep costs'!$F$1:$K$1,1,B18)))</f>
         <v/>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -957,19 +957,19 @@
         <v>0.1</v>
       </c>
       <c r="B5" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A5,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -978,19 +978,19 @@
         <v>0.5</v>
       </c>
       <c r="B6" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A6,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -999,19 +999,19 @@
         <v>1</v>
       </c>
       <c r="B7" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A7,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -1020,19 +1020,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A8,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -1041,19 +1041,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A9,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -1062,19 +1062,19 @@
         <v>10</v>
       </c>
       <c r="B10" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;B$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;C$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;D$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$17,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$17,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
+        <f>IFERROR(INDEX('Sweep costs'!$F$2:$K$25,MATCH(Pricer!$B$5&amp;"|ALL3|"&amp;E$4,'Sweep costs'!$A$2:$A$25,0),MATCH($A10,'Sweep costs'!$F$1:$K$1,0))+Pricer!$B$11,"not measured")</f>
         <v/>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1758,31 +1758,31 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>207</v>
+        <v>301</v>
       </c>
       <c r="F2" t="n">
         <v>0.001</v>
       </c>
       <c r="G2" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="H2" t="n">
-        <v>0.328</v>
+        <v>0.332</v>
       </c>
       <c r="I2" t="n">
-        <v>0.715</v>
+        <v>0.721</v>
       </c>
       <c r="J2" t="n">
-        <v>1.732</v>
+        <v>1.747</v>
       </c>
       <c r="K2" t="n">
-        <v>3.165</v>
+        <v>3.214</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BTC|ALL3|New York afternoon</t>
+          <t>BTC|ALL3|London morning</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1797,35 +1797,35 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>New York afternoon</t>
+          <t>London morning</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="F3" t="n">
         <v>0.001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.137</v>
+        <v>0.153</v>
       </c>
       <c r="H3" t="n">
-        <v>0.314</v>
+        <v>0.344</v>
       </c>
       <c r="I3" t="n">
-        <v>0.698</v>
+        <v>0.738</v>
       </c>
       <c r="J3" t="n">
-        <v>1.693</v>
+        <v>1.874</v>
       </c>
       <c r="K3" t="n">
-        <v>3.114</v>
+        <v>3.482</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BTC|binance|All measured</t>
+          <t>BTC|ALL3|New York afternoon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1835,40 +1835,40 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>binance</t>
+          <t>ALL3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>All measured</t>
+          <t>New York afternoon</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>207</v>
+        <v>164</v>
       </c>
       <c r="F4" t="n">
         <v>0.001</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.137</v>
       </c>
       <c r="H4" t="n">
-        <v>0.965</v>
+        <v>0.314</v>
       </c>
       <c r="I4" t="n">
-        <v>1.677</v>
+        <v>0.698</v>
       </c>
       <c r="J4" t="n">
-        <v>3.513</v>
+        <v>1.693</v>
       </c>
       <c r="K4" t="n">
-        <v>6.642</v>
+        <v>3.114</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BTC|binance|New York afternoon</t>
+          <t>BTC|binance|All measured</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1883,35 +1883,35 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New York afternoon</t>
+          <t>All measured</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>164</v>
+        <v>301</v>
       </c>
       <c r="F5" t="n">
         <v>0.001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>0.985</v>
+        <v>0.955</v>
       </c>
       <c r="I5" t="n">
-        <v>1.709</v>
+        <v>1.677</v>
       </c>
       <c r="J5" t="n">
-        <v>3.559</v>
+        <v>3.53</v>
       </c>
       <c r="K5" t="n">
-        <v>6.675</v>
+        <v>6.654</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BTC|coinbase|All measured</t>
+          <t>BTC|binance|London morning</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1921,40 +1921,40 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>coinbase</t>
+          <t>binance</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>All measured</t>
+          <t>London morning</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>207</v>
+        <v>137</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.014</v>
       </c>
       <c r="G6" t="n">
-        <v>1.65</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>2.256</v>
+        <v>0.915</v>
       </c>
       <c r="I6" t="n">
-        <v>3.563</v>
+        <v>1.625</v>
       </c>
       <c r="J6" t="n">
-        <v>7.639</v>
+        <v>3.483</v>
       </c>
       <c r="K6" t="n">
-        <v>13.218</v>
+        <v>6.612</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BTC|coinbase|New York afternoon</t>
+          <t>BTC|binance|New York afternoon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>coinbase</t>
+          <t>binance</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1976,28 +1976,28 @@
         <v>164</v>
       </c>
       <c r="F7" t="n">
-        <v>0.802</v>
+        <v>0.001</v>
       </c>
       <c r="G7" t="n">
-        <v>1.589</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>2.185</v>
+        <v>0.985</v>
       </c>
       <c r="I7" t="n">
-        <v>3.47</v>
+        <v>1.709</v>
       </c>
       <c r="J7" t="n">
-        <v>7.517</v>
+        <v>3.559</v>
       </c>
       <c r="K7" t="n">
-        <v>13.039</v>
+        <v>6.675</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BTC|kraken|All measured</t>
+          <t>BTC|coinbase|All measured</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kraken</t>
+          <t>coinbase</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2016,31 +2016,31 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>207</v>
+        <v>301</v>
       </c>
       <c r="F8" t="n">
-        <v>0.211</v>
+        <v>0.865</v>
       </c>
       <c r="G8" t="n">
-        <v>0.386</v>
+        <v>1.753</v>
       </c>
       <c r="H8" t="n">
-        <v>0.704</v>
+        <v>2.472</v>
       </c>
       <c r="I8" t="n">
-        <v>1.638</v>
+        <v>4.023</v>
       </c>
       <c r="J8" t="n">
-        <v>4.02</v>
+        <v>8.237</v>
       </c>
       <c r="K8" t="n">
-        <v>7.977</v>
+        <v>13.96</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BTC|kraken|New York afternoon</t>
+          <t>BTC|coinbase|London morning</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2050,179 +2050,179 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kraken</t>
+          <t>coinbase</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>New York afternoon</t>
+          <t>London morning</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="F9" t="n">
-        <v>0.158</v>
+        <v>0.973</v>
       </c>
       <c r="G9" t="n">
-        <v>0.368</v>
+        <v>2.098</v>
       </c>
       <c r="H9" t="n">
-        <v>0.658</v>
+        <v>3.212</v>
       </c>
       <c r="I9" t="n">
-        <v>1.564</v>
+        <v>5.35</v>
       </c>
       <c r="J9" t="n">
-        <v>3.953</v>
+        <v>10.99</v>
       </c>
       <c r="K9" t="n">
-        <v>7.837</v>
+        <v>18.442</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ETH|ALL3|All measured</t>
+          <t>BTC|coinbase|New York afternoon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ALL3</t>
+          <t>coinbase</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>All measured</t>
+          <t>New York afternoon</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>207</v>
+        <v>164</v>
       </c>
       <c r="F10" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.802</v>
       </c>
       <c r="G10" t="n">
-        <v>0.844</v>
+        <v>1.589</v>
       </c>
       <c r="H10" t="n">
-        <v>1.489</v>
+        <v>2.185</v>
       </c>
       <c r="I10" t="n">
-        <v>2.444</v>
+        <v>3.47</v>
       </c>
       <c r="J10" t="n">
-        <v>4.624</v>
+        <v>7.517</v>
       </c>
       <c r="K10" t="n">
-        <v>8.042</v>
+        <v>13.039</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ETH|ALL3|New York afternoon</t>
+          <t>BTC|kraken|All measured</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ALL3</t>
+          <t>kraken</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York afternoon</t>
+          <t>All measured</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>164</v>
+        <v>301</v>
       </c>
       <c r="F11" t="n">
-        <v>0.08</v>
+        <v>0.183</v>
       </c>
       <c r="G11" t="n">
-        <v>0.822</v>
+        <v>0.399</v>
       </c>
       <c r="H11" t="n">
-        <v>1.449</v>
+        <v>0.706</v>
       </c>
       <c r="I11" t="n">
-        <v>2.369</v>
+        <v>1.66</v>
       </c>
       <c r="J11" t="n">
-        <v>4.516</v>
+        <v>4.071</v>
       </c>
       <c r="K11" t="n">
-        <v>7.898</v>
+        <v>7.969</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ETH|binance|All measured</t>
+          <t>BTC|kraken|London morning</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>binance</t>
+          <t>kraken</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>All measured</t>
+          <t>London morning</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>207</v>
+        <v>137</v>
       </c>
       <c r="F12" t="n">
-        <v>0.181</v>
+        <v>0.214</v>
       </c>
       <c r="G12" t="n">
-        <v>1.356</v>
+        <v>0.447</v>
       </c>
       <c r="H12" t="n">
-        <v>2.471</v>
+        <v>0.785</v>
       </c>
       <c r="I12" t="n">
-        <v>4.308</v>
+        <v>1.781</v>
       </c>
       <c r="J12" t="n">
-        <v>9.363</v>
+        <v>4.259</v>
       </c>
       <c r="K12" t="n">
-        <v>36.27</v>
+        <v>8.089</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ETH|binance|New York afternoon</t>
+          <t>BTC|kraken|New York afternoon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>binance</t>
+          <t>kraken</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2234,28 +2234,28 @@
         <v>164</v>
       </c>
       <c r="F13" t="n">
-        <v>0.202</v>
+        <v>0.158</v>
       </c>
       <c r="G13" t="n">
-        <v>1.347</v>
+        <v>0.368</v>
       </c>
       <c r="H13" t="n">
-        <v>2.417</v>
+        <v>0.658</v>
       </c>
       <c r="I13" t="n">
-        <v>4.238</v>
+        <v>1.564</v>
       </c>
       <c r="J13" t="n">
-        <v>9.179</v>
+        <v>3.953</v>
       </c>
       <c r="K13" t="n">
-        <v>37.289</v>
+        <v>7.837</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ETH|coinbase|All measured</t>
+          <t>ETH|ALL3|All measured</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>coinbase</t>
+          <t>ALL3</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2274,31 +2274,31 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>207</v>
+        <v>301</v>
       </c>
       <c r="F14" t="n">
-        <v>1.405</v>
+        <v>0.062</v>
       </c>
       <c r="G14" t="n">
-        <v>4.009</v>
+        <v>0.86</v>
       </c>
       <c r="H14" t="n">
-        <v>6.549</v>
+        <v>1.52</v>
       </c>
       <c r="I14" t="n">
-        <v>10.63</v>
+        <v>2.519</v>
       </c>
       <c r="J14" t="n">
-        <v>21.793</v>
+        <v>4.806</v>
       </c>
       <c r="K14" t="n">
-        <v>85.21299999999999</v>
+        <v>8.375</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ETH|coinbase|New York afternoon</t>
+          <t>ETH|ALL3|London morning</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2308,40 +2308,40 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>coinbase</t>
+          <t>ALL3</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>New York afternoon</t>
+          <t>London morning</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="F15" t="n">
-        <v>1.368</v>
+        <v>0.036</v>
       </c>
       <c r="G15" t="n">
-        <v>3.907</v>
+        <v>0.916</v>
       </c>
       <c r="H15" t="n">
-        <v>6.363</v>
+        <v>1.618</v>
       </c>
       <c r="I15" t="n">
-        <v>10.433</v>
+        <v>2.714</v>
       </c>
       <c r="J15" t="n">
-        <v>21.527</v>
+        <v>5.004</v>
       </c>
       <c r="K15" t="n">
-        <v>83.48</v>
+        <v>8.832000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ETH|kraken|All measured</t>
+          <t>ETH|ALL3|New York afternoon</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2351,81 +2351,425 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>kraken</t>
+          <t>ALL3</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>All measured</t>
+          <t>New York afternoon</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>207</v>
+        <v>164</v>
       </c>
       <c r="F16" t="n">
-        <v>1.024</v>
+        <v>0.08</v>
       </c>
       <c r="G16" t="n">
-        <v>2.089</v>
+        <v>0.822</v>
       </c>
       <c r="H16" t="n">
-        <v>3.039</v>
+        <v>1.449</v>
       </c>
       <c r="I16" t="n">
-        <v>4.509</v>
+        <v>2.369</v>
       </c>
       <c r="J16" t="n">
-        <v>9.673999999999999</v>
+        <v>4.516</v>
       </c>
       <c r="K16" t="n">
-        <v>20.028</v>
+        <v>7.898</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>ETH|binance|All measured</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>binance</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>All measured</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>301</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.376</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2.517</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.448</v>
+      </c>
+      <c r="J17" t="n">
+        <v>9.811</v>
+      </c>
+      <c r="K17" t="n">
+        <v>37.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ETH|binance|London morning</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>binance</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>London morning</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>137</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.449</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.611</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4.666</v>
+      </c>
+      <c r="J18" t="n">
+        <v>10.558</v>
+      </c>
+      <c r="K18" t="n">
+        <v>36.855</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ETH|binance|New York afternoon</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>binance</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>New York afternoon</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>164</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.347</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2.417</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.238</v>
+      </c>
+      <c r="J19" t="n">
+        <v>9.179</v>
+      </c>
+      <c r="K19" t="n">
+        <v>37.289</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ETH|coinbase|All measured</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>coinbase</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>All measured</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>301</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.495</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4.044</v>
+      </c>
+      <c r="H20" t="n">
+        <v>6.775</v>
+      </c>
+      <c r="I20" t="n">
+        <v>10.849</v>
+      </c>
+      <c r="J20" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="K20" t="n">
+        <v>91.05500000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ETH|coinbase|London morning</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>coinbase</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>London morning</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>137</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.624</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4.176</v>
+      </c>
+      <c r="H21" t="n">
+        <v>7.129</v>
+      </c>
+      <c r="I21" t="n">
+        <v>11.554</v>
+      </c>
+      <c r="J21" t="n">
+        <v>32.455</v>
+      </c>
+      <c r="K21" t="n">
+        <v>128.529</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ETH|coinbase|New York afternoon</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>coinbase</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>New York afternoon</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>164</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3.907</v>
+      </c>
+      <c r="H22" t="n">
+        <v>6.363</v>
+      </c>
+      <c r="I22" t="n">
+        <v>10.433</v>
+      </c>
+      <c r="J22" t="n">
+        <v>21.527</v>
+      </c>
+      <c r="K22" t="n">
+        <v>83.48</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ETH|kraken|All measured</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>kraken</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>All measured</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>301</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.077</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.291</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3.264</v>
+      </c>
+      <c r="I23" t="n">
+        <v>4.716</v>
+      </c>
+      <c r="J23" t="n">
+        <v>9.996</v>
+      </c>
+      <c r="K23" t="n">
+        <v>20.46</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ETH|kraken|London morning</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>kraken</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>London morning</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>137</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.206</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2.579</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3.554</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4.928</v>
+      </c>
+      <c r="J24" t="n">
+        <v>10.426</v>
+      </c>
+      <c r="K24" t="n">
+        <v>21.297</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>ETH|kraken|New York afternoon</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>ETH</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>kraken</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>New York afternoon</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E25" t="n">
         <v>164</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F25" t="n">
         <v>0.968</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G25" t="n">
         <v>2.016</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H25" t="n">
         <v>2.925</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I25" t="n">
         <v>4.402</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J25" t="n">
         <v>9.484</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K25" t="n">
         <v>19.844</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Median cost of sweeping the displayed book, bps vs the venue's own mid, average of buy and sell. Columns are clip sizes in M$.</t>
         </is>
@@ -5634,7 +5978,7 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Sweep costs: 207 one-minute snapshots of the Binance (BTCUSDT, ETHUSDT), Coinbase and Kraken (BTC-USD, ETH-USD) books, 12 Oct 17:23 to 13 Oct 07:54 UTC.</t>
+          <t>Sweep costs: 301 one-minute snapshots of the Binance (BTCUSDT, ETHUSDT), Coinbase and Kraken (BTC-USD, ETH-USD) books, 12 Oct 17:23 to 13 Oct 09:28 UTC.</t>
         </is>
       </c>
     </row>

</xml_diff>